<commit_message>
Train a Skill: grades from the Level 1 Upper Skills sheet
Phase = the sheet's grade (0 = every phase). Sheet grades 4+ sit in
Phase 3, highlighted yellow for coach review. Standards and
prescriptions unchanged (finished templates).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015yWLLpzw9R1iGhMPWXgZsW
</commit_message>
<xml_diff>
--- a/Train_A_Skill/Level1_Skill_Horizontal_BentArmPull_RingPullFeetElevated.xlsx
+++ b/Train_A_Skill/Level1_Skill_Horizontal_BentArmPull_RingPullFeetElevated.xlsx
@@ -539,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -643,22 +643,22 @@
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>○  1</t>
+          <t>○  0</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Incline Archer Row</t>
+          <t>Single Arm DB Row</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>10 reps each arm at a 45° angle</t>
+          <t>10 reps at 35% bodyweight</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>6–10 reps</t>
+          <t>5–10 reps @ 10–15% BW</t>
         </is>
       </c>
     </row>
@@ -670,46 +670,23 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Single Arm DB Row</t>
+          <t>Chest Supported DB Row</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>10 reps at 35% bodyweight</t>
+          <t>10 reps with 60% bodyweight (total, both hands)</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>5–10 reps @ 10–15% BW</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>○  0</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Chest Supported DB Row</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>10 reps with 60% bodyweight (total, both hands)</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
           <t>5–10 reps @ 25–40% BW</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="D11:F11"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="A5:F5"/>
@@ -724,7 +701,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -802,17 +778,17 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Bent Leg Horizontal Row Isometric Hold</t>
+          <t>Incline Archer Row</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>30s hold at a horizontal angle</t>
+          <t>10 reps each arm at a 45° angle</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>15–30s</t>
+          <t>6–10 reps</t>
         </is>
       </c>
     </row>
@@ -824,17 +800,17 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Bent Leg Horizontal Rows</t>
+          <t>Bent Leg Horizontal Row Isometric Hold</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>15 reps</t>
+          <t>30s hold at a horizontal angle</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>5–15 reps</t>
+          <t>15–30s</t>
         </is>
       </c>
     </row>
@@ -846,17 +822,17 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Incline Bent Leg Single Arm Row</t>
+          <t>Bent Leg Horizontal Rows</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>10 reps each arm · body at a 45° angle, legs bent</t>
+          <t>15 reps</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>6–10 reps</t>
+          <t>5–15 reps</t>
         </is>
       </c>
     </row>
@@ -935,7 +911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1000,17 +976,17 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Ground Row Isometric Hold</t>
+          <t>Incline Bent Leg Single Arm Row</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>30s hold at a horizontal angle</t>
+          <t>10 reps each arm · body at a 45° angle, legs bent</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>15–30s</t>
+          <t>6–10 reps</t>
         </is>
       </c>
     </row>
@@ -1022,39 +998,39 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Ground Row</t>
+          <t>Ground Row Isometric Hold</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>12 reps</t>
+          <t>30s hold at a horizontal angle</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>6–12 reps</t>
+          <t>15–30s</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>○  0</t>
+          <t>○  3</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Single Arm DB Row</t>
+          <t>Ground Row</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>10 reps at 35% bodyweight</t>
+          <t>12 reps</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>5–10 reps @ 30–35% BW</t>
+          <t>6–12 reps</t>
         </is>
       </c>
     </row>
@@ -1066,23 +1042,46 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
+          <t>Single Arm DB Row</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>10 reps at 35% bodyweight</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>5–10 reps @ 30–35% BW</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>○  0</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
           <t>Chest Supported DB Row</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>10 reps with 60% bodyweight (total, both hands)</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>5–10 reps @ 55–60% BW</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="D11:F11"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="A5:F5"/>
@@ -1097,6 +1096,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>